<commit_message>
Excel using Python Updated
</commit_message>
<xml_diff>
--- a/Excel/Data.xlsx
+++ b/Excel/Data.xlsx
@@ -7,7 +7,7 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Data1" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -122,6 +122,19 @@
     </indexedColors>
   </colors>
 </styleSheet>
+</file>
+
+<file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Employee_Table" displayName="Employee_Table" ref="A1:D1" headerRowCount="1">
+  <autoFilter ref="A1:D1"/>
+  <tableColumns count="4">
+    <tableColumn id="1" name="None"/>
+    <tableColumn id="2" name="None"/>
+    <tableColumn id="3" name="None"/>
+    <tableColumn id="4" name="None"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="1"/>
+</table>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -417,5 +430,8 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <tableParts count="1">
+    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+  </tableParts>
 </worksheet>
 </file>
</xml_diff>